<commit_message>
Update Executive Dashboard Excel file with enhancements
</commit_message>
<xml_diff>
--- a/Executive_Dashboard.xlsx
+++ b/Executive_Dashboard.xlsx
@@ -32,7 +32,7 @@
     <numFmt numFmtId="168" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="169" formatCode="0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +58,45 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00102C5E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00102C5E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00102C5E"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -84,8 +121,20 @@
         <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7F0FF"/>
+        <bgColor rgb="00E7F0FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+        <bgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -99,11 +148,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -161,6 +238,32 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -705,729 +808,1637 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:W27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EXECUTIVE DASHBOARD - AT A GLANCE (2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Key Performance Indicators</t>
+          <t>CHII EXECUTIVE DASHBOARD - AT A GLANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Quarterly Trends (2022-2026) | Data Source: CHII MELA Consolidated Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>OUTREACH &amp; ACCESS METRICS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>2024 Actual</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
-        <is>
-          <t>2025 Target</t>
-        </is>
-      </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>2026 Target</t>
-        </is>
-      </c>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>Current (Q3)</t>
-        </is>
-      </c>
-      <c r="F4" s="20" t="inlineStr">
-        <is>
-          <t>Achievement %</t>
-        </is>
-      </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="n"/>
+      <c r="D4" s="30" t="n"/>
+      <c r="E4" s="31" t="n"/>
+      <c r="F4" s="37" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="n"/>
+      <c r="H4" s="30" t="n"/>
+      <c r="I4" s="31" t="n"/>
+      <c r="J4" s="37" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="K4" s="30" t="n"/>
+      <c r="L4" s="30" t="n"/>
+      <c r="M4" s="31" t="n"/>
+      <c r="N4" s="37" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="O4" s="30" t="n"/>
+      <c r="P4" s="30" t="n"/>
+      <c r="Q4" s="31" t="n"/>
+      <c r="R4" s="37" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="S4" s="30" t="n"/>
+      <c r="T4" s="30" t="n"/>
+      <c r="U4" s="31" t="n"/>
+      <c r="V4" s="36" t="inlineStr">
+        <is>
+          <t>2026 YoY %</t>
+        </is>
+      </c>
+      <c r="W4" s="36" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Total Participants Reached</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>38000</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>42000</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>45000</v>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>45320</v>
-      </c>
-      <c r="F5" s="21">
-        <f>E5/D5*100</f>
-        <v/>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>HEMP, HENT, HECO combined</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Total Ventures in Portfolio</t>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="G5" s="38" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="H5" s="38" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="I5" s="38" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="J5" s="38" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="K5" s="38" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="L5" s="38" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="M5" s="38" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="N5" s="38" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="O5" s="38" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="P5" s="38" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="Q5" s="38" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="R5" s="38" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S5" s="38" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="T5" s="38" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="U5" s="38" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Total Beneficiaries</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>82</v>
+        <v>180</v>
       </c>
       <c r="C6" s="8" t="n">
+        <v>320</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>520</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>720</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>850</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>980</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>1100</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>1150</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>1240</v>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="P6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="Q6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="R6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="S6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="T6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="U6" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="V6" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W6" s="25" t="inlineStr">
+        <is>
+          <t>Total across HEMP, HENT, HECO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Currently Enrolled</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="D7" s="8" t="n">
         <v>88</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="F6" s="21">
-        <f>E6/D6*100</f>
-        <v/>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>Across 5 cohorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Revenue-Generating Ventures (%)</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="n">
-        <v>55</v>
-      </c>
-      <c r="C7" s="22" t="n">
-        <v>62</v>
-      </c>
-      <c r="D7" s="22" t="n">
-        <v>70</v>
-      </c>
-      <c r="E7" s="22" t="n">
-        <v>67</v>
-      </c>
-      <c r="F7" s="21">
-        <f>E7/D7*100</f>
-        <v/>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>% of total ventures</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Total Funding Raised (USD M)</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="C8" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" s="23" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="E8" s="23" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="F8" s="21">
-        <f>E8/D8*100</f>
-        <v/>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>External + HENT funded</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Total Jobs Created</t>
+      <c r="E7" s="8" t="n">
+        <v>128</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>185</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>205</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>225</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>245</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>275</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="P7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="Q7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="R7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="S7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="T7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="U7" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="V7" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W7" s="25" t="inlineStr">
+        <is>
+          <t>Active programme participants</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>Graduates</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>145</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>215</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>310</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>520</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>680</v>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>730</v>
+      </c>
+      <c r="M8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="O8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="P8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="Q8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="R8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="S8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="T8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="U8" s="8" t="n">
+        <v>793</v>
+      </c>
+      <c r="V8" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W8" s="25" t="inlineStr">
+        <is>
+          <t>Programme completers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Youth with Disability</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>920</v>
+        <v>4</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>1050</v>
+        <v>8</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1200</v>
+        <v>12</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>1245</v>
-      </c>
-      <c r="F9" s="21">
-        <f>E9/D9*100</f>
-        <v/>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>Cumulative across ventures</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Employment Rate (%)</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="K9" s="8" t="n">
         <v>58</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="L9" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="D10" s="22" t="n">
-        <v>70</v>
-      </c>
-      <c r="E10" s="22" t="n">
+      <c r="M9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="P9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="Q9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="R9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="S9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="T9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="U9" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="V9" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W9" s="25" t="inlineStr">
+        <is>
+          <t>PWD participants</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Refugee / IDP</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" s="8" t="n">
         <v>68</v>
       </c>
-      <c r="F10" s="21">
-        <f>E10/D10*100</f>
-        <v/>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>% of graduates employed</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Women-led Ventures (%)</t>
-        </is>
-      </c>
-      <c r="B11" s="22" t="n">
+      <c r="H10" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>128</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>135</v>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="O10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="P10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="Q10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="R10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="S10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="T10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="U10" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="V10" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W10" s="25" t="inlineStr">
+        <is>
+          <t>Displaced population support</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>MCF Scholars</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>480</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>520</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>535</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>544</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="P11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="Q11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="R11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="S11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="T11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="U11" s="8" t="n">
+        <v>552</v>
+      </c>
+      <c r="V11" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W11" s="25" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation scholars</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>CSAT Score (0-5)</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="Q12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="R12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="S12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="T12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="U12" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="V12" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W12" s="25" t="inlineStr">
+        <is>
+          <t>Customer satisfaction (n=240)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Employer Rating (0-5)</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="N13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="P13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="Q13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="R13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="S13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="T13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="U13" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="V13" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="W13" s="25" t="inlineStr">
+        <is>
+          <t>Employer feedback (n=156)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>PROGRAM OUTCOMES - YOUTH IN WORK &amp; EMPLOYMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>Youth in Work (Total)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>112</v>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>126</v>
+      </c>
+      <c r="L15" s="8" t="n">
+        <v>129</v>
+      </c>
+      <c r="M15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="P15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="Q15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="R15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="S15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="T15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="U15" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="V15" s="10" t="inlineStr">
+        <is>
+          <t>+8%</t>
+        </is>
+      </c>
+      <c r="W15" s="40" t="inlineStr">
+        <is>
+          <t>Active workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>Wage Employment</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="K16" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="L16" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="N16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="O16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="P16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="Q16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="R16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="S16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="T16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="U16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="V16" s="10" t="inlineStr">
+        <is>
+          <t>+12%</t>
+        </is>
+      </c>
+      <c r="W16" s="40" t="inlineStr">
+        <is>
+          <t>Employed (wage jobs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>Entrepreneurs</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="O17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="P17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="R17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="S17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="T17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="U17" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="V17" s="10" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="W17" s="40" t="inlineStr">
+        <is>
+          <t>Business owners</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>Jobs Created (Total)</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>520</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>850</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>1220</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>1750</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>1920</v>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v>2050</v>
+      </c>
+      <c r="K18" s="8" t="n">
+        <v>2090</v>
+      </c>
+      <c r="L18" s="8" t="n">
+        <v>2120</v>
+      </c>
+      <c r="M18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="N18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="O18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="P18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="Q18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="R18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="S18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="T18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="U18" s="8" t="n">
+        <v>2151</v>
+      </c>
+      <c r="V18" s="10" t="inlineStr">
+        <is>
+          <t>+18%</t>
+        </is>
+      </c>
+      <c r="W18" s="40" t="inlineStr">
+        <is>
+          <t>Direct employment created</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>Active Ventures</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="O19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="P19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="R19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="S19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="T19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="U19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="V19" s="10" t="inlineStr">
+        <is>
+          <t>+22%</t>
+        </is>
+      </c>
+      <c r="W19" s="40" t="inlineStr">
+        <is>
+          <t>Enterprises generating revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="39" t="inlineStr">
+        <is>
+          <t>Freelancers</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="J20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="K20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="L20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="M20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="N20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="O20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="P20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="R20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="S20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="T20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="U20" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="V20" s="10" t="inlineStr">
+        <is>
+          <t>-3%</t>
+        </is>
+      </c>
+      <c r="W20" s="40" t="inlineStr">
+        <is>
+          <t>Self-employed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>Job Seeking</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="L21" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="C11" s="22" t="n">
-        <v>38</v>
-      </c>
-      <c r="D11" s="22" t="n">
-        <v>42</v>
-      </c>
-      <c r="E11" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="F11" s="21">
-        <f>E11/D11*100</f>
-        <v/>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>% of venture portfolio</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Female Participant Rate (%)</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="n">
-        <v>48</v>
-      </c>
-      <c r="C12" s="22" t="n">
+      <c r="M21" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="N21" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="22" t="n">
-        <v>55</v>
-      </c>
-      <c r="E12" s="22" t="n">
+      <c r="O21" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="P21" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q21" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="R21" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="S21" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="T21" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="U21" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="V21" s="10" t="inlineStr">
+        <is>
+          <t>-15%</t>
+        </is>
+      </c>
+      <c r="W21" s="40" t="inlineStr">
+        <is>
+          <t>In transition / seeking</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="39" t="inlineStr">
+        <is>
+          <t>Continuing Studies</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="D22" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="F12" s="21">
-        <f>E12/D12*100</f>
-        <v/>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>All programmes combined</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Health System Actors (Count)</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="D13" s="8" t="n">
+      <c r="E22" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="F22" s="8" t="n">
         <v>110</v>
       </c>
-      <c r="E13" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="F13" s="21">
-        <f>E13/D13*100</f>
-        <v/>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>Using HENT solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Lives Impacted (Est. Count)</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>180000</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>220000</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>288000</v>
-      </c>
-      <c r="F14" s="21">
-        <f>E14/D14*100</f>
-        <v/>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>By HENT health innovations</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Active Research Partnerships</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="F15" s="21">
-        <f>E15/D15*100</f>
-        <v/>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>Formal MOUs signed</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Policy Changes Influenced</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" s="21">
-        <f>E16/D16*100</f>
-        <v/>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>Government adopted</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Performance Summary by Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="24" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B19" s="24" t="inlineStr">
-        <is>
-          <t>Target Achievement</t>
-        </is>
-      </c>
-      <c r="C19" s="24" t="inlineStr">
-        <is>
-          <t>vs. 2025</t>
-        </is>
-      </c>
-      <c r="D19" s="24" t="inlineStr">
-        <is>
-          <t>Quarterly Progress</t>
-        </is>
-      </c>
-      <c r="E19" s="24" t="inlineStr">
-        <is>
-          <t>Key Insight</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>Reach &amp; Participation</t>
-        </is>
-      </c>
-      <c r="B20" s="26" t="inlineStr">
-        <is>
-          <t>100.7%</t>
-        </is>
-      </c>
-      <c r="C20" s="27" t="inlineStr">
-        <is>
-          <t>+3.3K participants</t>
-        </is>
-      </c>
-      <c r="D20" s="27" t="inlineStr">
-        <is>
-          <t>Q3: 34.5K cumulative</t>
-        </is>
-      </c>
-      <c r="E20" s="25" t="inlineStr">
-        <is>
-          <t>Strong growth across all pillars</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="25" t="inlineStr">
-        <is>
-          <t>Venture Portfolio</t>
-        </is>
-      </c>
-      <c r="B21" s="26" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="C21" s="27" t="inlineStr">
-        <is>
-          <t>8 new ventures</t>
-        </is>
-      </c>
-      <c r="D21" s="27" t="inlineStr">
-        <is>
-          <t>On track for year-end</t>
-        </is>
-      </c>
-      <c r="E21" s="25" t="inlineStr">
-        <is>
-          <t>Stable cohort pipeline</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="25" t="inlineStr">
-        <is>
-          <t>Employment Outcomes</t>
-        </is>
-      </c>
-      <c r="B22" s="26" t="inlineStr">
-        <is>
-          <t>97%</t>
-        </is>
-      </c>
-      <c r="C22" s="27" t="inlineStr">
-        <is>
-          <t>+205 jobs</t>
-        </is>
-      </c>
-      <c r="D22" s="27" t="inlineStr">
-        <is>
-          <t>Q3: 980 placed</t>
-        </is>
-      </c>
-      <c r="E22" s="25" t="inlineStr">
-        <is>
-          <t>Wage employment driving growth</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>Funding Mobilization</t>
-        </is>
-      </c>
-      <c r="B23" s="26" t="inlineStr">
-        <is>
-          <t>96.5%</t>
-        </is>
-      </c>
-      <c r="C23" s="27" t="inlineStr">
-        <is>
-          <t>+1.2M USD</t>
-        </is>
-      </c>
-      <c r="D23" s="27" t="inlineStr">
-        <is>
-          <t>Q3: 6.8M mobilized</t>
-        </is>
-      </c>
-      <c r="E23" s="25" t="inlineStr">
-        <is>
-          <t>External funding increasing</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="25" t="inlineStr">
-        <is>
-          <t>Health System Impact</t>
-        </is>
-      </c>
-      <c r="B24" s="26" t="inlineStr">
-        <is>
-          <t>96%</t>
-        </is>
-      </c>
-      <c r="C24" s="27" t="inlineStr">
-        <is>
-          <t>+16 new actors</t>
-        </is>
-      </c>
-      <c r="D24" s="27" t="inlineStr">
-        <is>
-          <t>Q3: 85 actors active</t>
-        </is>
-      </c>
-      <c r="E24" s="25" t="inlineStr">
-        <is>
-          <t>Policy adoption accelerating</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Quarterly Progress (2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B27" s="24" t="inlineStr">
-        <is>
-          <t>Q1 Actual</t>
-        </is>
-      </c>
-      <c r="C27" s="24" t="inlineStr">
-        <is>
-          <t>Q2 Actual</t>
-        </is>
-      </c>
-      <c r="D27" s="24" t="inlineStr">
-        <is>
-          <t>Q3 Actual</t>
-        </is>
-      </c>
-      <c r="E27" s="24" t="inlineStr">
-        <is>
-          <t>Q4 Target</t>
-        </is>
-      </c>
-      <c r="F27" s="24" t="inlineStr">
-        <is>
-          <t>Full Year Target</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Participants (Cumulative)</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="n">
-        <v>10500</v>
-      </c>
-      <c r="C28" s="8" t="n">
-        <v>22800</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <v>34500</v>
-      </c>
-      <c r="E28" s="8" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F28" s="8" t="n">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>New Ventures Identified</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="C29" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="D29" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>36</v>
-      </c>
-      <c r="F29" s="8" t="n">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Employment Placements</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="n">
-        <v>340</v>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>680</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>980</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F30" s="8" t="n">
-        <v>1245</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Funding Mobilized (USD M)</t>
-        </is>
-      </c>
-      <c r="B31" s="23" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="C31" s="23" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D31" s="23" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="E31" s="23" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="F31" s="23" t="n">
-        <v>8.199999999999999</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Health Actors Reached</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>58</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>110</v>
-      </c>
-      <c r="F32" s="8" t="n">
-        <v>101</v>
-      </c>
+      <c r="G22" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>185</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="S22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="T22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="U22" s="8" t="n">
+        <v>206</v>
+      </c>
+      <c r="V22" s="10" t="inlineStr">
+        <is>
+          <t>+11%</t>
+        </is>
+      </c>
+      <c r="W22" s="40" t="inlineStr">
+        <is>
+          <t>Further education pursuits</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="35" t="inlineStr">
+        <is>
+          <t>KEY PERFORMANCE INSIGHTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>Gender Balance</t>
+        </is>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>Female participants (Target: 50%)</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="n"/>
+      <c r="E24" s="40" t="inlineStr">
+        <is>
+          <t>Exceeds target across all programmes</t>
+        </is>
+      </c>
+      <c r="F24" s="30" t="n"/>
+      <c r="G24" s="30" t="n"/>
+      <c r="H24" s="30" t="n"/>
+      <c r="I24" s="30" t="n"/>
+      <c r="J24" s="30" t="n"/>
+      <c r="K24" s="30" t="n"/>
+      <c r="L24" s="30" t="n"/>
+      <c r="M24" s="30" t="n"/>
+      <c r="N24" s="30" t="n"/>
+      <c r="O24" s="30" t="n"/>
+      <c r="P24" s="30" t="n"/>
+      <c r="Q24" s="30" t="n"/>
+      <c r="R24" s="30" t="n"/>
+      <c r="S24" s="30" t="n"/>
+      <c r="T24" s="30" t="n"/>
+      <c r="U24" s="31" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>+28%</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>Regional Growth</t>
+        </is>
+      </c>
+      <c r="C25" s="40" t="inlineStr">
+        <is>
+          <t>YoY expansion across 12 countries</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="n"/>
+      <c r="E25" s="40" t="inlineStr">
+        <is>
+          <t>East Africa +38%, West Africa activated</t>
+        </is>
+      </c>
+      <c r="F25" s="30" t="n"/>
+      <c r="G25" s="30" t="n"/>
+      <c r="H25" s="30" t="n"/>
+      <c r="I25" s="30" t="n"/>
+      <c r="J25" s="30" t="n"/>
+      <c r="K25" s="30" t="n"/>
+      <c r="L25" s="30" t="n"/>
+      <c r="M25" s="30" t="n"/>
+      <c r="N25" s="30" t="n"/>
+      <c r="O25" s="30" t="n"/>
+      <c r="P25" s="30" t="n"/>
+      <c r="Q25" s="30" t="n"/>
+      <c r="R25" s="30" t="n"/>
+      <c r="S25" s="30" t="n"/>
+      <c r="T25" s="30" t="n"/>
+      <c r="U25" s="31" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="B26" s="39" t="inlineStr">
+        <is>
+          <t>Employment Success</t>
+        </is>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>Graduate employment rate</t>
+        </is>
+      </c>
+      <c r="D26" s="31" t="n"/>
+      <c r="E26" s="40" t="inlineStr">
+        <is>
+          <t>Wage 39%, Self-emp 23%, Further ed 14%</t>
+        </is>
+      </c>
+      <c r="F26" s="30" t="n"/>
+      <c r="G26" s="30" t="n"/>
+      <c r="H26" s="30" t="n"/>
+      <c r="I26" s="30" t="n"/>
+      <c r="J26" s="30" t="n"/>
+      <c r="K26" s="30" t="n"/>
+      <c r="L26" s="30" t="n"/>
+      <c r="M26" s="30" t="n"/>
+      <c r="N26" s="30" t="n"/>
+      <c r="O26" s="30" t="n"/>
+      <c r="P26" s="30" t="n"/>
+      <c r="Q26" s="30" t="n"/>
+      <c r="R26" s="30" t="n"/>
+      <c r="S26" s="30" t="n"/>
+      <c r="T26" s="30" t="n"/>
+      <c r="U26" s="31" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B27" s="39" t="inlineStr">
+        <is>
+          <t>Venture Momentum</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>New enterprises (↑22% YoY)</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="40" t="inlineStr">
+        <is>
+          <t>2,151 jobs created, avg $52K revenue</t>
+        </is>
+      </c>
+      <c r="F27" s="30" t="n"/>
+      <c r="G27" s="30" t="n"/>
+      <c r="H27" s="30" t="n"/>
+      <c r="I27" s="30" t="n"/>
+      <c r="J27" s="30" t="n"/>
+      <c r="K27" s="30" t="n"/>
+      <c r="L27" s="30" t="n"/>
+      <c r="M27" s="30" t="n"/>
+      <c r="N27" s="30" t="n"/>
+      <c r="O27" s="30" t="n"/>
+      <c r="P27" s="30" t="n"/>
+      <c r="Q27" s="30" t="n"/>
+      <c r="R27" s="30" t="n"/>
+      <c r="S27" s="30" t="n"/>
+      <c r="T27" s="30" t="n"/>
+      <c r="U27" s="31" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="18">
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="R4:U4"/>
+    <mergeCell ref="E26:U26"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="E25:U25"/>
+    <mergeCell ref="A14:U14"/>
+    <mergeCell ref="E24:U24"/>
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A23:U23"/>
+    <mergeCell ref="E27:U27"/>
+    <mergeCell ref="A3:U3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2515,9 +3526,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A3:E3"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>